<commit_message>
feat: implement quest system with progress tracking and completion
- Add quest class with luable inheritance and Lua binding support
- Implement character quest management functions (quest, start_quest, remove_quest, can_start_quest)
- Add quest object builtin functions (model, progress, step, inc_progress, inc_step, complete, completed)
- Create quest model builtin functions (step, progress, reward)
- Add quest and reward data tables
- Update character class with quest-related methods
- Integrate quest system with existing game architecture
</commit_message>
<xml_diff>
--- a/resources/table/reward.xlsx
+++ b/resources/table/reward.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cshyeon\fb\resources\table\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\fb\resources\table\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4DF1F2B-931B-42A8-9573-F482BD948E29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3674330D-4391-46D0-863A-5E86D43E9824}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17790" xr2:uid="{D06B357D-EBE0-49AC-A207-4E89A5AA0593}"/>
+    <workbookView xWindow="38280" yWindow="-135" windowWidth="38640" windowHeight="21120" xr2:uid="{D06B357D-EBE0-49AC-A207-4E89A5AA0593}"/>
   </bookViews>
   <sheets>
     <sheet name="reward" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="8">
   <si>
     <t>id</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -44,6 +44,18 @@
   </si>
   <si>
     <t>[dsl]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>quest1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>quest1.step.1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>quest1.step.3</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -107,7 +119,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="표준" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -123,9 +135,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 테마">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -163,7 +175,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -269,7 +281,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -411,7 +423,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -419,10 +431,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE8D9647-70DB-4352-ABD3-4D2F60838B15}">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="16384" width="9" style="1"/>
+    <col min="1" max="1" width="11.375" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
@@ -449,6 +462,21 @@
         <v>2</v>
       </c>
     </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>